<commit_message>
Cleanup reqs + add provided docs Wagga
</commit_message>
<xml_diff>
--- a/docs/provided/wagga/EXP 2 design and Session structure_MJB.xlsx
+++ b/docs/provided/wagga/EXP 2 design and Session structure_MJB.xlsx
@@ -5,12 +5,12 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Structure" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="TrialOrder" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="Trial_Events_Log_Audio" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Trial_EventSequence" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="299" uniqueCount="116">
   <si>
     <t xml:space="preserve">Session info</t>
   </si>
@@ -243,45 +243,12 @@
     <t xml:space="preserve">Randomised (R)esponse / (N)o (R)esponse Schedule</t>
   </si>
   <si>
+    <t xml:space="preserve">Q. Are there 2 lots of trials on day 6 – what about Day 7?</t>
+  </si>
+  <si>
     <t xml:space="preserve">iTrial</t>
   </si>
   <si>
-    <t xml:space="preserve">Day 1: 7 / 0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Day 1: 3 / 0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Day 2: 3 / 0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Day 2: 7 / 0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Day 3: 7 / 0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Day 3: 3 / 0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Day 4: 3 / 0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Day 4: 7 / 0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Day 5: 3 / 0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Day 5: 7 / 0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Day 6: 7 / 0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Day 7: 3 / 0</t>
-  </si>
-  <si>
     <t xml:space="preserve">R</t>
   </si>
   <si>
@@ -303,10 +270,19 @@
     <t xml:space="preserve">Trainer 2 High</t>
   </si>
   <si>
+    <t xml:space="preserve">Understanding Sequence of events?</t>
+  </si>
+  <si>
     <t xml:space="preserve">Questions</t>
   </si>
   <si>
-    <t xml:space="preserve">Is nTrial fixed at 10? (Believe it is)</t>
+    <t xml:space="preserve">Is nTrial fixed at 10? (TODO: Confirm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">For each trial (iTrial = 1 to 10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ref #</t>
   </si>
   <si>
     <t xml:space="preserve">Trial Stage</t>
@@ -321,10 +297,7 @@
     <t xml:space="preserve">Audio output</t>
   </si>
   <si>
-    <t xml:space="preserve">For each trial (iTrial = 1 to 10)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Is this any specific button (e.g. green)?</t>
+    <t xml:space="preserve">Is this any specific button (e.g. green)? Only one button?</t>
   </si>
   <si>
     <t xml:space="preserve">Initiation</t>
@@ -336,19 +309,22 @@
     <t xml:space="preserve">Is this the one sound or ten different sounds?</t>
   </si>
   <si>
+    <t xml:space="preserve">Start trial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Time of button press = StartTime</t>
+  </si>
+  <si>
     <t xml:space="preserve">Reward/No-reward</t>
   </si>
   <si>
     <t xml:space="preserve">Dispensing of any reward</t>
   </si>
   <si>
-    <t xml:space="preserve">Does this happen here or later?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Start trial</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Time of button press = StartTime</t>
+    <t xml:space="preserve">Reward" OR "No reward</t>
+  </si>
+  <si>
+    <t xml:space="preserve">When does reward happen?</t>
   </si>
   <si>
     <t xml:space="preserve">Response period</t>
@@ -360,7 +336,7 @@
     <t xml:space="preserve">Count cumulative responses</t>
   </si>
   <si>
-    <t xml:space="preserve">How is each response measured?</t>
+    <t xml:space="preserve">Confirm how is each response measured? Just one time difference?</t>
   </si>
   <si>
     <t xml:space="preserve">Termination</t>
@@ -369,10 +345,31 @@
     <t xml:space="preserve">Is there a button press here?</t>
   </si>
   <si>
-    <t xml:space="preserve">Elapsed time between trials – not recorded – can be implied from difference of EndTime and Start/Initiation of next trial</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Don’t need to record?</t>
+    <t xml:space="preserve">More questions?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Is there just 1 type of experiment or 2? i.e. just CB or other?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What if there are interruptions? Errors?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Just restart trial? Re-use trial number or new trial number e.g. nTrial is number of successful trials?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Elapsed time between trials – not recorded – can be implied from difference of EndTime and Start/Initiation of next trial?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Do you need to record which trainer (or this is implied from schedule)? e.g. make one of start-up parameters</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Robot = RaspberryPi? Why restarts?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WiFi available this time?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Do you want to confirm the system time before experiments?</t>
   </si>
 </sst>
 </file>
@@ -383,7 +380,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="@"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="12">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -446,8 +443,29 @@
       <family val="2"/>
       <charset val="1"/>
     </font>
+    <font>
+      <b val="true"/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -460,8 +478,26 @@
         <bgColor rgb="FFCCCCFF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFB2B2B2"/>
+        <bgColor rgb="FFB4C7DC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEEEEEE"/>
+        <bgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor rgb="FFEEEEEE"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="7">
+  <borders count="12">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
@@ -511,6 +547,65 @@
       <bottom style="thin"/>
       <diagonal/>
     </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin">
+        <color rgb="FF666666"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF666666"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF666666"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF666666"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right style="thin">
+        <color rgb="FF666666"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF666666"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF666666"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin"/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin">
+        <color rgb="FF666666"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF666666"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF666666"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right style="thin">
+        <color rgb="FF666666"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF666666"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="20">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -537,104 +632,188 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="46">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="10" fillId="3" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="3" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="3" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="11" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="11" fillId="4" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="4" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="4" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="11" fillId="5" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="5" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="5" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -667,7 +846,7 @@
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFFFFFCC"/>
+      <rgbColor rgb="FFEEEEEE"/>
       <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
@@ -695,8 +874,8 @@
       <rgbColor rgb="FFFFCC00"/>
       <rgbColor rgb="FFFF9900"/>
       <rgbColor rgb="FFFF6600"/>
-      <rgbColor rgb="FF666699"/>
-      <rgbColor rgb="FF969696"/>
+      <rgbColor rgb="FF666666"/>
+      <rgbColor rgb="FFB2B2B2"/>
       <rgbColor rgb="FF003366"/>
       <rgbColor rgb="FF339966"/>
       <rgbColor rgb="FF003300"/>
@@ -721,9 +900,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>950400</xdr:colOff>
+      <xdr:colOff>950040</xdr:colOff>
       <xdr:row>39</xdr:row>
-      <xdr:rowOff>104400</xdr:rowOff>
+      <xdr:rowOff>104040</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -737,7 +916,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="1536840" y="6156360"/>
-          <a:ext cx="6140880" cy="2377800"/>
+          <a:ext cx="6140880" cy="2377440"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -758,9 +937,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
-      <xdr:colOff>1066680</xdr:colOff>
+      <xdr:colOff>1066320</xdr:colOff>
       <xdr:row>38</xdr:row>
-      <xdr:rowOff>126720</xdr:rowOff>
+      <xdr:rowOff>126360</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -773,8 +952,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="9659160" y="6019920"/>
-          <a:ext cx="6126840" cy="2336400"/>
+          <a:off x="9659880" y="6019920"/>
+          <a:ext cx="6126480" cy="2336040"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -969,369 +1148,369 @@
   <dimension ref="A1:L41"/>
   <sheetFormatPr defaultColWidth="10.46875" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="21.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="3" style="0" width="14.84"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="18.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="23.34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="19"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="15.5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="26.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="22.34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="21.66"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="3" style="1" width="14.84"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="18.66"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="23.34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="15.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="26.66"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="22.34"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="0" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="0" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="0" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="0" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="0" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="0" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="0" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="E2" s="0" t="s">
+      <c r="E2" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="F2" s="0" t="s">
+      <c r="F2" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="G2" s="0" t="s">
+      <c r="G2" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="H2" s="0" t="s">
+      <c r="H2" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="I2" s="0" t="s">
+      <c r="I2" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J2" s="0" t="s">
+      <c r="J2" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="K2" s="0" t="s">
+      <c r="K2" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="L2" s="0" t="s">
+      <c r="L2" s="1" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="I3" s="0" t="s">
+      <c r="I3" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="J3" s="0" t="s">
+      <c r="J3" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="K3" s="0" t="s">
+      <c r="K3" s="1" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+      <c r="A4" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="J4" s="0" t="s">
+      <c r="J4" s="1" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+      <c r="A5" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" s="2" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="2" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
+      <c r="A7" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" s="2" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
+      <c r="A8" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B8" s="2" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="1" t="s">
+      <c r="B9" s="2" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="33.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="s">
+      <c r="A10" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" s="2" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="1" t="s">
+      <c r="B11" s="2" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="33.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="1" t="s">
+      <c r="B12" s="2" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="1" t="s">
+      <c r="B13" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="C13" s="0" t="s">
+      <c r="C13" s="1" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C14" s="0" t="s">
+      <c r="C14" s="1" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C15" s="0" t="s">
+      <c r="C15" s="1" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C17" s="0" t="s">
+      <c r="C17" s="1" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="18" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="1" t="s">
+      <c r="B21" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="C21" s="0" t="s">
+      <c r="C21" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="D21" s="0" t="s">
+      <c r="D21" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="E21" s="0" t="s">
+      <c r="E21" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="F21" s="0" t="s">
+      <c r="F21" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="G21" s="0" t="s">
+      <c r="G21" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="H21" s="0" t="s">
+      <c r="H21" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="I21" s="0" t="s">
+      <c r="I21" s="1" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="3" t="s">
+      <c r="A22" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="B22" s="4" t="s">
+      <c r="B22" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="C22" s="4" t="s">
+      <c r="C22" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="D22" s="4" t="s">
+      <c r="D22" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="E22" s="4" t="s">
+      <c r="E22" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="F22" s="4" t="s">
+      <c r="F22" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="G22" s="4" t="s">
+      <c r="G22" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="H22" s="4" t="s">
+      <c r="H22" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="I22" s="4" t="s">
+      <c r="I22" s="5" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="5" t="s">
+      <c r="A23" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="B23" s="6" t="s">
+      <c r="B23" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="C23" s="6" t="s">
+      <c r="C23" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="D23" s="6" t="s">
+      <c r="D23" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="E23" s="6" t="s">
+      <c r="E23" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="F23" s="6" t="s">
+      <c r="F23" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="G23" s="6" t="s">
+      <c r="G23" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="H23" s="6" t="s">
+      <c r="H23" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="I23" s="6" t="s">
+      <c r="I23" s="7" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="7" t="s">
+      <c r="A24" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="B24" s="8" t="s">
+      <c r="B24" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="C24" s="6" t="s">
+      <c r="C24" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="D24" s="6" t="s">
+      <c r="D24" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="E24" s="6" t="s">
+      <c r="E24" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="F24" s="6" t="s">
+      <c r="F24" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="G24" s="6" t="s">
+      <c r="G24" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="H24" s="6" t="s">
+      <c r="H24" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="I24" s="8" t="s">
+      <c r="I24" s="9" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="8" t="s">
+      <c r="A25" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="B25" s="8"/>
-      <c r="C25" s="8" t="s">
+      <c r="B25" s="9"/>
+      <c r="C25" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="D25" s="8" t="s">
+      <c r="D25" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="E25" s="8" t="s">
+      <c r="E25" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="F25" s="8" t="s">
+      <c r="F25" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="G25" s="9" t="s">
+      <c r="G25" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="H25" s="8" t="s">
+      <c r="H25" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="I25" s="8"/>
+      <c r="I25" s="9"/>
     </row>
     <row r="26" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="8"/>
-      <c r="B26" s="8"/>
-      <c r="C26" s="8"/>
-      <c r="D26" s="8"/>
-      <c r="E26" s="8"/>
-      <c r="F26" s="8"/>
-      <c r="G26" s="6" t="s">
+      <c r="A26" s="9"/>
+      <c r="B26" s="9"/>
+      <c r="C26" s="9"/>
+      <c r="D26" s="9"/>
+      <c r="E26" s="9"/>
+      <c r="F26" s="9"/>
+      <c r="G26" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="H26" s="8"/>
-      <c r="I26" s="8"/>
+      <c r="H26" s="9"/>
+      <c r="I26" s="9"/>
     </row>
     <row r="28" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="0" t="s">
+      <c r="A28" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="G28" s="0" t="s">
+      <c r="G28" s="1" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B41" s="1" t="s">
+      <c r="B41" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="C41" s="0" t="s">
+      <c r="C41" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="E41" s="0" t="s">
+      <c r="E41" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="H41" s="1" t="s">
+      <c r="H41" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="I41" s="0" t="s">
+      <c r="I41" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="K41" s="0" t="s">
+      <c r="K41" s="1" t="s">
         <v>70</v>
       </c>
     </row>
@@ -1362,679 +1541,732 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M22"/>
+  <dimension ref="A1:N22"/>
   <sheetFormatPr defaultColWidth="10.46875" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6.84"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="6.84"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="21.4"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="10"/>
-      <c r="B1" s="11" t="s">
+      <c r="A1" s="11"/>
+      <c r="B1" s="12" t="s">
         <v>72</v>
       </c>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
-      <c r="G1" s="12"/>
-      <c r="H1" s="12"/>
-      <c r="I1" s="12"/>
-      <c r="J1" s="12"/>
-      <c r="K1" s="12"/>
-      <c r="L1" s="12"/>
-      <c r="M1" s="12"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="13"/>
+      <c r="I1" s="13"/>
+      <c r="J1" s="13"/>
+      <c r="K1" s="13"/>
+      <c r="L1" s="13"/>
+      <c r="M1" s="13"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="10"/>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
-      <c r="F2" s="12"/>
-      <c r="G2" s="12"/>
-      <c r="H2" s="12"/>
-      <c r="I2" s="12"/>
-      <c r="J2" s="12"/>
-      <c r="K2" s="12"/>
-      <c r="L2" s="12"/>
-      <c r="M2" s="12"/>
+      <c r="A2" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="B2" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="13" t="n">
+        <f aca="false">B2</f>
+        <v>1</v>
+      </c>
+      <c r="D2" s="13" t="n">
+        <f aca="false">B2+1</f>
+        <v>2</v>
+      </c>
+      <c r="E2" s="13" t="n">
+        <f aca="false">D2</f>
+        <v>2</v>
+      </c>
+      <c r="F2" s="13" t="n">
+        <f aca="false">D2+1</f>
+        <v>3</v>
+      </c>
+      <c r="G2" s="13" t="n">
+        <f aca="false">F2</f>
+        <v>3</v>
+      </c>
+      <c r="H2" s="13" t="n">
+        <f aca="false">F2+1</f>
+        <v>4</v>
+      </c>
+      <c r="I2" s="13" t="n">
+        <f aca="false">H2</f>
+        <v>4</v>
+      </c>
+      <c r="J2" s="13" t="n">
+        <f aca="false">H2+1</f>
+        <v>5</v>
+      </c>
+      <c r="K2" s="13" t="n">
+        <f aca="false">J2</f>
+        <v>5</v>
+      </c>
+      <c r="L2" s="13" t="n">
+        <f aca="false">J2+1</f>
+        <v>6</v>
+      </c>
+      <c r="M2" s="13" t="n">
+        <f aca="false">L2</f>
+        <v>6</v>
+      </c>
+      <c r="N2" s="14" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="13" t="s">
-        <v>73</v>
-      </c>
-      <c r="B3" s="14" t="s">
+      <c r="A3" s="15" t="s">
         <v>74</v>
       </c>
-      <c r="C3" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="D3" s="14" t="s">
-        <v>76</v>
-      </c>
-      <c r="E3" s="14" t="s">
+      <c r="B3" s="16" t="str">
+        <f aca="false">"Day " &amp; B2 &amp; ": " &amp; B14 &amp; " / " &amp; 10-B14</f>
+        <v>Day 1: 7 / 3</v>
+      </c>
+      <c r="C3" s="16" t="str">
+        <f aca="false">"Day " &amp; C2 &amp; ": " &amp; C14 &amp; " / " &amp; 10-C14</f>
+        <v>Day 1: 3 / 7</v>
+      </c>
+      <c r="D3" s="16" t="str">
+        <f aca="false">"Day " &amp; D2 &amp; ": " &amp; D14 &amp; " / " &amp; 10-D14</f>
+        <v>Day 2: 3 / 7</v>
+      </c>
+      <c r="E3" s="16" t="str">
+        <f aca="false">"Day " &amp; E2 &amp; ": " &amp; E14 &amp; " / " &amp; 10-E14</f>
+        <v>Day 2: 7 / 3</v>
+      </c>
+      <c r="F3" s="16" t="str">
+        <f aca="false">"Day " &amp; F2 &amp; ": " &amp; F14 &amp; " / " &amp; 10-F14</f>
+        <v>Day 3: 7 / 3</v>
+      </c>
+      <c r="G3" s="16" t="str">
+        <f aca="false">"Day " &amp; G2 &amp; ": " &amp; G14 &amp; " / " &amp; 10-G14</f>
+        <v>Day 3: 3 / 7</v>
+      </c>
+      <c r="H3" s="16" t="str">
+        <f aca="false">"Day " &amp; H2 &amp; ": " &amp; H14 &amp; " / " &amp; 10-H14</f>
+        <v>Day 4: 3 / 7</v>
+      </c>
+      <c r="I3" s="16" t="str">
+        <f aca="false">"Day " &amp; I2 &amp; ": " &amp; I14 &amp; " / " &amp; 10-I14</f>
+        <v>Day 4: 7 / 3</v>
+      </c>
+      <c r="J3" s="16" t="str">
+        <f aca="false">"Day " &amp; J2 &amp; ": " &amp; J14 &amp; " / " &amp; 10-J14</f>
+        <v>Day 5: 3 / 7</v>
+      </c>
+      <c r="K3" s="16" t="str">
+        <f aca="false">"Day " &amp; K2 &amp; ": " &amp; K14 &amp; " / " &amp; 10-K14</f>
+        <v>Day 5: 7 / 3</v>
+      </c>
+      <c r="L3" s="16" t="str">
+        <f aca="false">"Day " &amp; L2 &amp; ": " &amp; L14 &amp; " / " &amp; 10-L14</f>
+        <v>Day 6: 7 / 3</v>
+      </c>
+      <c r="M3" s="16" t="str">
+        <f aca="false">"Day " &amp; M2 &amp; ": " &amp; M14 &amp; " / " &amp; 10-M14</f>
+        <v>Day 6: 3 / 7</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="C4" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="D4" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="E4" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="F4" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="G4" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="H4" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="I4" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="J4" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="K4" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="L4" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="M4" s="17" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="C5" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="D5" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="E5" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="F5" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="G5" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="H5" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="I5" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="J5" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="K5" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="L5" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="M5" s="17" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="C6" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="D6" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="E6" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="F6" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="G6" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="H6" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="I6" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="J6" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="K6" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="L6" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="M6" s="17" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="C7" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="D7" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="E7" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="F7" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="G7" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="H7" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="I7" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="J7" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="K7" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="L7" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="M7" s="17" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="C8" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="D8" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="E8" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="F8" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="G8" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="H8" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="I8" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="J8" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="K8" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="L8" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="M8" s="17" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="15" t="n">
+        <v>6</v>
+      </c>
+      <c r="B9" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="C9" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="D9" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="E9" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="F9" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="G9" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="H9" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="I9" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="J9" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="K9" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="L9" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="M9" s="17" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="B10" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="C10" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="D10" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="E10" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="F10" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="G10" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="H10" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="I10" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="J10" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="K10" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="L10" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="M10" s="17" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="B11" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="C11" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="D11" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="E11" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="F11" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="G11" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="H11" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="I11" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="J11" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="K11" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="L11" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="M11" s="17" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="15" t="n">
+        <v>9</v>
+      </c>
+      <c r="B12" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="C12" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="D12" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="E12" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="F12" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="G12" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="H12" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="I12" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="J12" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="K12" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="L12" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="M12" s="17" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="B13" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="C13" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="D13" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="E13" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="F13" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="G13" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="H13" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="I13" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="J13" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="K13" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="L13" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="M13" s="17" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="18" t="s">
         <v>77</v>
       </c>
-      <c r="F3" s="14" t="s">
-        <v>78</v>
-      </c>
-      <c r="G3" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="H3" s="14" t="s">
-        <v>80</v>
-      </c>
-      <c r="I3" s="14" t="s">
-        <v>81</v>
-      </c>
-      <c r="J3" s="14" t="s">
-        <v>82</v>
-      </c>
-      <c r="K3" s="14" t="s">
-        <v>83</v>
-      </c>
-      <c r="L3" s="14" t="s">
-        <v>84</v>
-      </c>
-      <c r="M3" s="14" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="B4" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="C4" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="D4" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="E4" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="F4" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="G4" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="H4" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="I4" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="J4" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="K4" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="L4" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="M4" s="15" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="13" t="n">
-        <v>2</v>
-      </c>
-      <c r="B5" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="C5" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="D5" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="E5" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="F5" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="G5" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="H5" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="I5" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="J5" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="K5" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="L5" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="M5" s="15" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="13" t="n">
-        <v>3</v>
-      </c>
-      <c r="B6" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="C6" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="D6" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="E6" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="F6" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="G6" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="H6" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="I6" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="J6" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="K6" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="L6" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="M6" s="15" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="13" t="n">
-        <v>4</v>
-      </c>
-      <c r="B7" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="C7" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="D7" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="E7" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="F7" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="G7" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="H7" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="I7" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="J7" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="K7" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="L7" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="M7" s="15" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="13" t="n">
-        <v>5</v>
-      </c>
-      <c r="B8" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="C8" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="D8" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="E8" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="F8" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="G8" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="H8" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="I8" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="J8" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="K8" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="L8" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="M8" s="15" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="13" t="n">
-        <v>6</v>
-      </c>
-      <c r="B9" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="C9" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="D9" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="E9" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="F9" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="G9" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="H9" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="I9" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="J9" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="K9" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="L9" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="M9" s="15" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="13" t="n">
-        <v>7</v>
-      </c>
-      <c r="B10" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="C10" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="D10" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="E10" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="F10" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="G10" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="H10" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="I10" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="J10" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="K10" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="L10" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="M10" s="15" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="13" t="n">
-        <v>8</v>
-      </c>
-      <c r="B11" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="C11" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="D11" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="E11" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="F11" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="G11" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="H11" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="I11" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="J11" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="K11" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="L11" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="M11" s="15" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="13" t="n">
-        <v>9</v>
-      </c>
-      <c r="B12" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="C12" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="D12" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="E12" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="F12" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="G12" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="H12" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="I12" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="J12" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="K12" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="L12" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="M12" s="15" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="13" t="n">
-        <v>10</v>
-      </c>
-      <c r="B13" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="C13" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="D13" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="E13" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="F13" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="G13" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="H13" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="I13" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="J13" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="K13" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="L13" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="M13" s="15" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="16" t="s">
-        <v>88</v>
-      </c>
-      <c r="B14" s="14" t="n">
+      <c r="B14" s="16" t="n">
         <f aca="false">COUNTIF(B4:B13,"R")</f>
         <v>7</v>
       </c>
-      <c r="C14" s="14" t="n">
+      <c r="C14" s="16" t="n">
         <f aca="false">COUNTIF(C4:C13,"R")</f>
         <v>3</v>
       </c>
-      <c r="D14" s="14" t="n">
+      <c r="D14" s="16" t="n">
         <f aca="false">COUNTIF(D4:D13,"R")</f>
         <v>3</v>
       </c>
-      <c r="E14" s="14" t="n">
+      <c r="E14" s="16" t="n">
         <f aca="false">COUNTIF(E4:E13,"R")</f>
         <v>7</v>
       </c>
-      <c r="F14" s="14" t="n">
+      <c r="F14" s="16" t="n">
         <f aca="false">COUNTIF(F4:F13,"R")</f>
         <v>7</v>
       </c>
-      <c r="G14" s="14" t="n">
+      <c r="G14" s="16" t="n">
         <f aca="false">COUNTIF(G4:G13,"R")</f>
         <v>3</v>
       </c>
-      <c r="H14" s="14" t="n">
+      <c r="H14" s="16" t="n">
         <f aca="false">COUNTIF(H4:H13,"R")</f>
         <v>3</v>
       </c>
-      <c r="I14" s="14" t="n">
+      <c r="I14" s="16" t="n">
         <f aca="false">COUNTIF(I4:I13,"R")</f>
         <v>7</v>
       </c>
-      <c r="J14" s="14" t="n">
+      <c r="J14" s="16" t="n">
         <f aca="false">COUNTIF(J4:J13,"R")</f>
         <v>3</v>
       </c>
-      <c r="K14" s="14" t="n">
+      <c r="K14" s="16" t="n">
         <f aca="false">COUNTIF(K4:K13,"R")</f>
         <v>7</v>
       </c>
-      <c r="L14" s="14" t="n">
+      <c r="L14" s="16" t="n">
         <f aca="false">COUNTIF(L4:L13,"R")</f>
         <v>7</v>
       </c>
-      <c r="M14" s="14" t="n">
+      <c r="M14" s="16" t="n">
         <f aca="false">COUNTIF(M4:M13,"R")</f>
         <v>3</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="17"/>
+      <c r="B15" s="19"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="17" t="s">
-        <v>89</v>
+      <c r="B16" s="20" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="18" customFormat="false" ht="22.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="18" t="s">
+      <c r="A18" s="21" t="s">
         <v>44</v>
       </c>
-      <c r="B18" s="19" t="s">
+      <c r="B18" s="22" t="s">
         <v>45</v>
       </c>
-      <c r="C18" s="19" t="s">
+      <c r="C18" s="22" t="s">
         <v>46</v>
       </c>
-      <c r="D18" s="19" t="s">
+      <c r="D18" s="22" t="s">
         <v>47</v>
       </c>
-      <c r="E18" s="19" t="s">
+      <c r="E18" s="22" t="s">
         <v>48</v>
       </c>
-      <c r="F18" s="19" t="s">
+      <c r="F18" s="22" t="s">
         <v>49</v>
       </c>
-      <c r="G18" s="19" t="s">
+      <c r="G18" s="22" t="s">
         <v>50</v>
       </c>
-      <c r="H18" s="19" t="s">
+      <c r="H18" s="22" t="s">
         <v>51</v>
       </c>
-      <c r="I18" s="19" t="s">
+      <c r="I18" s="22" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="22.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="18" t="s">
-        <v>90</v>
-      </c>
-      <c r="B19" s="20" t="s">
+      <c r="A19" s="21" t="s">
+        <v>79</v>
+      </c>
+      <c r="B19" s="23" t="s">
         <v>54</v>
       </c>
-      <c r="C19" s="20" t="s">
+      <c r="C19" s="23" t="s">
         <v>55</v>
       </c>
-      <c r="D19" s="20" t="s">
+      <c r="D19" s="23" t="s">
         <v>55</v>
       </c>
-      <c r="E19" s="20" t="s">
+      <c r="E19" s="23" t="s">
         <v>55</v>
       </c>
-      <c r="F19" s="20" t="s">
+      <c r="F19" s="23" t="s">
         <v>55</v>
       </c>
-      <c r="G19" s="20" t="s">
+      <c r="G19" s="23" t="s">
         <v>56</v>
       </c>
-      <c r="H19" s="20" t="s">
-        <v>91</v>
-      </c>
-      <c r="I19" s="20" t="s">
+      <c r="H19" s="23" t="s">
+        <v>80</v>
+      </c>
+      <c r="I19" s="23" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="21" t="s">
+      <c r="A20" s="24" t="s">
         <v>59</v>
       </c>
-      <c r="B20" s="21" t="s">
+      <c r="B20" s="24" t="s">
         <v>60</v>
       </c>
-      <c r="C20" s="20" t="s">
+      <c r="C20" s="23" t="s">
         <v>61</v>
       </c>
-      <c r="D20" s="20" t="s">
+      <c r="D20" s="23" t="s">
         <v>62</v>
       </c>
-      <c r="E20" s="20" t="s">
+      <c r="E20" s="23" t="s">
         <v>61</v>
       </c>
-      <c r="F20" s="20" t="s">
+      <c r="F20" s="23" t="s">
         <v>62</v>
       </c>
-      <c r="G20" s="20" t="s">
+      <c r="G20" s="23" t="s">
         <v>63</v>
       </c>
-      <c r="H20" s="20" t="s">
+      <c r="H20" s="23" t="s">
         <v>61</v>
       </c>
-      <c r="I20" s="21" t="s">
+      <c r="I20" s="24" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="21" t="s">
+      <c r="A21" s="24" t="s">
         <v>65</v>
       </c>
-      <c r="B21" s="21"/>
-      <c r="C21" s="20" t="s">
+      <c r="B21" s="24"/>
+      <c r="C21" s="23" t="s">
         <v>62</v>
       </c>
-      <c r="D21" s="20" t="s">
+      <c r="D21" s="23" t="s">
         <v>66</v>
       </c>
-      <c r="E21" s="20" t="s">
+      <c r="E21" s="23" t="s">
         <v>62</v>
       </c>
-      <c r="F21" s="20" t="s">
+      <c r="F21" s="23" t="s">
         <v>61</v>
       </c>
-      <c r="G21" s="20" t="s">
-        <v>92</v>
-      </c>
-      <c r="H21" s="20" t="s">
+      <c r="G21" s="23" t="s">
+        <v>81</v>
+      </c>
+      <c r="H21" s="23" t="s">
         <v>62</v>
       </c>
-      <c r="I21" s="21"/>
+      <c r="I21" s="24"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="21"/>
-      <c r="B22" s="21"/>
-      <c r="C22" s="20"/>
-      <c r="D22" s="20"/>
-      <c r="E22" s="20"/>
-      <c r="F22" s="20"/>
-      <c r="G22" s="20"/>
-      <c r="H22" s="20"/>
-      <c r="I22" s="21"/>
+      <c r="A22" s="24"/>
+      <c r="B22" s="24"/>
+      <c r="C22" s="23"/>
+      <c r="D22" s="23"/>
+      <c r="E22" s="23"/>
+      <c r="F22" s="23"/>
+      <c r="G22" s="23"/>
+      <c r="H22" s="23"/>
+      <c r="I22" s="24"/>
     </row>
   </sheetData>
   <mergeCells count="9">
@@ -2063,136 +2295,221 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
-  <sheetFormatPr defaultColWidth="10.4921875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:G22"/>
+  <sheetFormatPr defaultColWidth="10.4921875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="20.74"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="21.99"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="33.59"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="25.74"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5.92"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="28.35"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="23.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="32.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="22.06"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="25" width="2.16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="37.48"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F1" s="22" t="s">
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="26" t="s">
+        <v>82</v>
+      </c>
+      <c r="G1" s="27" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B2" s="0"/>
+      <c r="C2" s="0"/>
+      <c r="D2" s="0"/>
+      <c r="E2" s="0"/>
+      <c r="F2" s="28"/>
+      <c r="G2" s="20" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B3" s="29" t="s">
+        <v>85</v>
+      </c>
+      <c r="C3" s="30"/>
+      <c r="D3" s="30"/>
+      <c r="E3" s="30"/>
+      <c r="G3" s="31"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="32" t="s">
+        <v>86</v>
+      </c>
+      <c r="B4" s="33" t="s">
+        <v>87</v>
+      </c>
+      <c r="C4" s="33" t="s">
+        <v>88</v>
+      </c>
+      <c r="D4" s="33" t="s">
+        <v>89</v>
+      </c>
+      <c r="E4" s="34" t="s">
+        <v>90</v>
+      </c>
+      <c r="F4" s="35"/>
+      <c r="G4" s="20" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="37" t="s">
+        <v>92</v>
+      </c>
+      <c r="C5" s="37" t="s">
+        <v>12</v>
+      </c>
+      <c r="D5" s="37" t="s">
         <v>93</v>
       </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F2" s="17" t="s">
+      <c r="E5" s="38" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" s="39"/>
+      <c r="G5" s="20" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B3" s="22" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="40" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="41" t="s">
         <v>95</v>
       </c>
-      <c r="C3" s="22" t="s">
+      <c r="C6" s="41" t="s">
+        <v>12</v>
+      </c>
+      <c r="D6" s="41" t="s">
         <v>96</v>
       </c>
-      <c r="D3" s="22" t="s">
+      <c r="E6" s="42"/>
+      <c r="F6" s="39"/>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="36" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="37" t="s">
         <v>97</v>
       </c>
-      <c r="E3" s="22" t="s">
+      <c r="C7" s="37" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="23" t="s">
+      <c r="D7" s="37" t="s">
+        <v>15</v>
+      </c>
+      <c r="E7" s="38" t="s">
         <v>99</v>
       </c>
-      <c r="B4" s="24"/>
-      <c r="C4" s="24"/>
-      <c r="D4" s="24"/>
-      <c r="E4" s="24"/>
-      <c r="F4" s="17" t="s">
+      <c r="F7" s="39"/>
+      <c r="G7" s="20" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="0" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="40" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="41" t="s">
         <v>101</v>
       </c>
-      <c r="C5" s="0" t="s">
+      <c r="C8" s="41" t="s">
+        <v>102</v>
+      </c>
+      <c r="D8" s="41" t="s">
+        <v>103</v>
+      </c>
+      <c r="E8" s="42"/>
+      <c r="F8" s="39"/>
+      <c r="G8" s="20" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="43" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="44" t="s">
+        <v>105</v>
+      </c>
+      <c r="C9" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="D5" s="0" t="s">
-        <v>102</v>
-      </c>
-      <c r="E5" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="F5" s="17" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="0" t="s">
-        <v>104</v>
-      </c>
-      <c r="C6" s="0" t="s">
-        <v>105</v>
-      </c>
-      <c r="D6" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="E6" s="0" t="s">
-        <v>16</v>
-      </c>
-      <c r="F6" s="17" t="s">
+      <c r="D9" s="44" t="s">
+        <v>18</v>
+      </c>
+      <c r="E9" s="45"/>
+      <c r="F9" s="39"/>
+      <c r="G9" s="20" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="0" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B10" s="0"/>
+      <c r="G10" s="20"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B11" s="0"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B13" s="0"/>
+      <c r="C13" s="0"/>
+      <c r="D13" s="0"/>
+      <c r="E13" s="0"/>
+      <c r="F13" s="28"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B14" s="27" t="s">
         <v>107</v>
       </c>
-      <c r="C7" s="0" t="s">
-        <v>12</v>
-      </c>
-      <c r="D7" s="0" t="s">
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B15" s="31" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B8" s="0" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B16" s="27" t="s">
         <v>109</v>
       </c>
-      <c r="C8" s="0" t="s">
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B17" s="27" t="s">
         <v>110</v>
       </c>
-      <c r="D8" s="0" t="s">
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B18" s="27" t="s">
         <v>111</v>
       </c>
-      <c r="F8" s="17" t="s">
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B19" s="27" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="0" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B20" s="27" t="s">
         <v>113</v>
       </c>
-      <c r="C9" s="0" t="s">
-        <v>12</v>
-      </c>
-      <c r="D9" s="0" t="s">
-        <v>18</v>
-      </c>
-      <c r="F9" s="17" t="s">
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B21" s="27" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="0" t="s">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B22" s="27" t="s">
         <v>115</v>
       </c>
-      <c r="F10" s="17" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>

</xml_diff>